<commit_message>
Finish finding Vertex Group Remap for Yelan
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/YelanRemapDraft.xlsx
+++ b/Data/RemapDrafts/YelanRemapDraft.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Computer\Games\Genshin\Repos\Repos\Fix-Raiden-Boss\Data\RemapDrafts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19838E65-7CE3-46B7-AFA7-CBB23F9A6C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F0206CD-1B1D-410C-814A-CC21E514264A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{188B206F-658D-4ECC-A5DF-0C850120EB3C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Uncertainty</t>
   </si>
@@ -60,6 +60,111 @@
   </si>
   <si>
     <t>YelanTranquilEye</t>
+  </si>
+  <si>
+    <t>Yelan's jacket, right  side</t>
+  </si>
+  <si>
+    <t>Yelan's jacket, left side</t>
+  </si>
+  <si>
+    <t>Yelan's hood</t>
+  </si>
+  <si>
+    <t>Yelans jacket back</t>
+  </si>
+  <si>
+    <t>Yelan's right fur</t>
+  </si>
+  <si>
+    <t>Yelan's left fur</t>
+  </si>
+  <si>
+    <t>Yelan's right earing</t>
+  </si>
+  <si>
+    <t>Yelan's left earing</t>
+  </si>
+  <si>
+    <t>Yelan's right back bang</t>
+  </si>
+  <si>
+    <t>Yelan's left back bang</t>
+  </si>
+  <si>
+    <t>Yelan's front left top dress</t>
+  </si>
+  <si>
+    <t>Yelan's left bangle</t>
+  </si>
+  <si>
+    <t>Yelans' back top dress</t>
+  </si>
+  <si>
+    <t>Yelan's back dress</t>
+  </si>
+  <si>
+    <t>Yelan's back right dress</t>
+  </si>
+  <si>
+    <t>Yelan's back left dress</t>
+  </si>
+  <si>
+    <t>Yelan's front top left dress</t>
+  </si>
+  <si>
+    <t>Yelan's dice tie</t>
+  </si>
+  <si>
+    <t>Yelan's fur thing dangling behind jacket</t>
+  </si>
+  <si>
+    <t>Yelan's right upper arm</t>
+  </si>
+  <si>
+    <t>Yelan's right middle arm</t>
+  </si>
+  <si>
+    <t>Yelan's left upper arm</t>
+  </si>
+  <si>
+    <t>Yelans's vision by her right waist</t>
+  </si>
+  <si>
+    <t>Yelan's head</t>
+  </si>
+  <si>
+    <t>Yelan's main right shoulder</t>
+  </si>
+  <si>
+    <t>Yelan's sub right shoulder</t>
+  </si>
+  <si>
+    <t>Yelan's sub left shoulder</t>
+  </si>
+  <si>
+    <t>Yelan's right foot</t>
+  </si>
+  <si>
+    <t>Yelan's right lower arm</t>
+  </si>
+  <si>
+    <t>Yelans' right thigh</t>
+  </si>
+  <si>
+    <t>Yelan's right toes</t>
+  </si>
+  <si>
+    <t>Yelan's left thigh</t>
+  </si>
+  <si>
+    <t>Yelan's main left shoulder</t>
+  </si>
+  <si>
+    <t>Yelan's left foot</t>
+  </si>
+  <si>
+    <t>Yelan's left lower arm</t>
   </si>
 </sst>
 </file>
@@ -110,7 +215,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -569,6 +684,9 @@
       <c r="E7">
         <v>0.5</v>
       </c>
+      <c r="F7" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -615,543 +733,985 @@
       <c r="A12">
         <v>10</v>
       </c>
+      <c r="B12">
+        <v>68</v>
+      </c>
+      <c r="E12">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
+      <c r="B13">
+        <v>68</v>
+      </c>
+      <c r="E13">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
+      <c r="B14">
+        <v>63</v>
+      </c>
+      <c r="E14">
+        <v>0.5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
+      <c r="B15">
+        <v>63</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>15</v>
+      </c>
+      <c r="E20">
+        <v>0.1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>39</v>
+      </c>
+      <c r="E21">
+        <v>0.1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>67</v>
+      </c>
+      <c r="E22">
+        <v>0.15</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>63</v>
+      </c>
+      <c r="F23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>65</v>
+      </c>
+      <c r="F24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B26">
+        <v>69</v>
+      </c>
+      <c r="E26">
+        <v>0.1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>82</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="D30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="D31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>85</v>
+      </c>
+      <c r="F33" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>83</v>
+      </c>
+      <c r="F35" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>35</v>
       </c>
-      <c r="D37">
+      <c r="C37">
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>36</v>
       </c>
-      <c r="D38">
+      <c r="C38">
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>37</v>
       </c>
-      <c r="D39">
+      <c r="C39">
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38</v>
       </c>
-      <c r="D40">
+      <c r="C40">
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>39</v>
       </c>
-      <c r="D41">
+      <c r="C41">
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>99</v>
+      </c>
+      <c r="E42">
+        <v>0.25</v>
+      </c>
+      <c r="F42" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>100</v>
+      </c>
+      <c r="E43">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>94</v>
+      </c>
+      <c r="E44">
+        <v>0.2</v>
+      </c>
+      <c r="F44" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>95</v>
+      </c>
+      <c r="E45">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>112</v>
+      </c>
+      <c r="F46" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B47">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <v>103</v>
+      </c>
+      <c r="F49" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <v>114</v>
+      </c>
+      <c r="F51" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>50</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>51</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B53">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>52</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B54">
+        <v>127</v>
+      </c>
+      <c r="F54" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>53</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B55">
+        <v>91</v>
+      </c>
+      <c r="F55" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>54</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <v>63</v>
+      </c>
+      <c r="F56" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>55</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <v>77</v>
+      </c>
+      <c r="E57">
+        <v>0.2</v>
+      </c>
+      <c r="F57" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>56</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B58">
+        <v>78</v>
+      </c>
+      <c r="E58">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>57</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B59">
+        <v>79</v>
+      </c>
+      <c r="E59">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>58</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B60">
+        <v>11</v>
+      </c>
+      <c r="F60" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>59</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B61">
+        <v>36</v>
+      </c>
+      <c r="F61" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>60</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B62">
+        <v>12</v>
+      </c>
+      <c r="F62" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>61</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B63">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>62</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B64">
+        <v>116</v>
+      </c>
+      <c r="F64" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>63</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B65">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>64</v>
       </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B66">
+        <v>13</v>
+      </c>
+      <c r="F66" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>65</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B67">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>66</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B68">
+        <v>15</v>
+      </c>
+      <c r="F68" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>67</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B69">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>68</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B70">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>69</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B71">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>70</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B72">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>71</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B73">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>72</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B74">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>73</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B75">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>74</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B76">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>75</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B77">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>76</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B78">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>77</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B79">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>78</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B80">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>79</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B81">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>80</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B82">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>81</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B83">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>82</v>
       </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B84">
+        <v>31</v>
+      </c>
+      <c r="F84" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>83</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B85">
+        <v>32</v>
+      </c>
+      <c r="F85" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>84</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B86">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>85</v>
       </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B87">
+        <v>34</v>
+      </c>
+      <c r="F87" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>86</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B88">
+        <v>35</v>
+      </c>
+      <c r="F88" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>87</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B89">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>88</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B90">
+        <v>38</v>
+      </c>
+      <c r="F90" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>89</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B91">
+        <v>39</v>
+      </c>
+      <c r="F91" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>90</v>
       </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B92">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>91</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B93">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>92</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B94">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>93</v>
       </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B95">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>94</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B96">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>95</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B97">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>96</v>
       </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B98">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>97</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B99">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>98</v>
       </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B100">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>99</v>
       </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B101">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>100</v>
       </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B102">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>101</v>
       </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B103">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>102</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B104">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>103</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B105">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>104</v>
       </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B106">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>105</v>
       </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B107">
+        <v>55</v>
+      </c>
+      <c r="F107" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>106</v>
       </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B108">
+        <v>56</v>
+      </c>
+      <c r="F108" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>107</v>
       </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B109">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>108</v>
       </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B110">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>109</v>
       </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B111">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>110</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B112">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>111</v>
       </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B113">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>112</v>
       </c>
+      <c r="B114">
+        <v>63</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F114" xr:uid="{141D28D4-55F4-4C77-9C10-EC02550CE7B6}"/>
-  <conditionalFormatting sqref="B2:D114">
+  <conditionalFormatting sqref="B2:B114">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C114">
     <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C37:C41">
+    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D2:D114">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>